<commit_message>
Practica 02: filtro de particulas implementado y reporte
</commit_message>
<xml_diff>
--- a/resultados_astar.xlsx
+++ b/resultados_astar.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J65"/>
+  <dimension ref="A1:J81"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="5" min="1" max="1"/>
@@ -2983,6 +2983,646 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" s="12" t="n">
+        <v>63</v>
+      </c>
+      <c r="B66" s="12" t="inlineStr">
+        <is>
+          <t>(-0.00, -0.00)</t>
+        </is>
+      </c>
+      <c r="C66" s="12" t="inlineStr">
+        <is>
+          <t>(3.91, 3.30)</t>
+        </is>
+      </c>
+      <c r="D66" s="12" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E66" s="12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F66" s="12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G66" s="12" t="n">
+        <v>26.45</v>
+      </c>
+      <c r="H66" s="12" t="n">
+        <v>78</v>
+      </c>
+      <c r="I66" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J66" s="12" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="B67" s="11" t="inlineStr">
+        <is>
+          <t>(3.59, 3.27)</t>
+        </is>
+      </c>
+      <c r="C67" s="11" t="inlineStr">
+        <is>
+          <t>(0.10, 0.10)</t>
+        </is>
+      </c>
+      <c r="D67" s="11" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E67" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F67" s="11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G67" s="11" t="n">
+        <v>16.04</v>
+      </c>
+      <c r="H67" s="11" t="n">
+        <v>70</v>
+      </c>
+      <c r="I67" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J67" s="11" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="12" t="n">
+        <v>65</v>
+      </c>
+      <c r="B68" s="12" t="inlineStr">
+        <is>
+          <t>(0.37, 0.10)</t>
+        </is>
+      </c>
+      <c r="C68" s="12" t="inlineStr">
+        <is>
+          <t>(3.51, 3.27)</t>
+        </is>
+      </c>
+      <c r="D68" s="12" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E68" s="12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F68" s="12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G68" s="12" t="n">
+        <v>4.28</v>
+      </c>
+      <c r="H68" s="12" t="n">
+        <v>63</v>
+      </c>
+      <c r="I68" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J68" s="12" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="11" t="n">
+        <v>66</v>
+      </c>
+      <c r="B69" s="11" t="inlineStr">
+        <is>
+          <t>(3.24, 3.08)</t>
+        </is>
+      </c>
+      <c r="C69" s="11" t="inlineStr">
+        <is>
+          <t>(4.68, 1.81)</t>
+        </is>
+      </c>
+      <c r="D69" s="11" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E69" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F69" s="11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G69" s="11" t="n">
+        <v>3.01</v>
+      </c>
+      <c r="H69" s="11" t="n">
+        <v>28</v>
+      </c>
+      <c r="I69" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J69" s="11" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="12" t="n">
+        <v>67</v>
+      </c>
+      <c r="B70" s="12" t="inlineStr">
+        <is>
+          <t>(-0.00, -0.00)</t>
+        </is>
+      </c>
+      <c r="C70" s="12" t="inlineStr">
+        <is>
+          <t>(3.83, 3.12)</t>
+        </is>
+      </c>
+      <c r="D70" s="12" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E70" s="12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F70" s="12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G70" s="12" t="n">
+        <v>26.79</v>
+      </c>
+      <c r="H70" s="12" t="n">
+        <v>76</v>
+      </c>
+      <c r="I70" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J70" s="12" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="11" t="n">
+        <v>68</v>
+      </c>
+      <c r="B71" s="11" t="inlineStr">
+        <is>
+          <t>(-0.00, 0.00)</t>
+        </is>
+      </c>
+      <c r="C71" s="11" t="inlineStr">
+        <is>
+          <t>(1.99, 2.75)</t>
+        </is>
+      </c>
+      <c r="D71" s="11" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E71" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F71" s="11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G71" s="11" t="n">
+        <v>19.19</v>
+      </c>
+      <c r="H71" s="11" t="n">
+        <v>55</v>
+      </c>
+      <c r="I71" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J71" s="11" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="12" t="n">
+        <v>69</v>
+      </c>
+      <c r="B72" s="12" t="inlineStr">
+        <is>
+          <t>(-0.00, -0.00)</t>
+        </is>
+      </c>
+      <c r="C72" s="12" t="inlineStr">
+        <is>
+          <t>(1.55, 3.26)</t>
+        </is>
+      </c>
+      <c r="D72" s="12" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E72" s="12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F72" s="12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G72" s="12" t="n">
+        <v>54.7</v>
+      </c>
+      <c r="H72" s="12" t="n">
+        <v>65</v>
+      </c>
+      <c r="I72" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J72" s="12" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="11" t="n">
+        <v>70</v>
+      </c>
+      <c r="B73" s="11" t="inlineStr">
+        <is>
+          <t>(-0.00, -0.00)</t>
+        </is>
+      </c>
+      <c r="C73" s="11" t="inlineStr">
+        <is>
+          <t>(0.99, 3.01)</t>
+        </is>
+      </c>
+      <c r="D73" s="11" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E73" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F73" s="11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G73" s="11" t="n">
+        <v>19.46</v>
+      </c>
+      <c r="H73" s="11" t="n">
+        <v>60</v>
+      </c>
+      <c r="I73" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J73" s="11" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="12" t="n">
+        <v>71</v>
+      </c>
+      <c r="B74" s="12" t="inlineStr">
+        <is>
+          <t>(-0.00, -0.00)</t>
+        </is>
+      </c>
+      <c r="C74" s="12" t="inlineStr">
+        <is>
+          <t>(1.03, 3.12)</t>
+        </is>
+      </c>
+      <c r="D74" s="12" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E74" s="12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F74" s="12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G74" s="12" t="n">
+        <v>30.99</v>
+      </c>
+      <c r="H74" s="12" t="n">
+        <v>63</v>
+      </c>
+      <c r="I74" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J74" s="12" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="11" t="n">
+        <v>72</v>
+      </c>
+      <c r="B75" s="11" t="inlineStr">
+        <is>
+          <t>(-0.00, -0.00)</t>
+        </is>
+      </c>
+      <c r="C75" s="11" t="inlineStr">
+        <is>
+          <t>(0.99, 3.07)</t>
+        </is>
+      </c>
+      <c r="D75" s="11" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E75" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F75" s="11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G75" s="11" t="n">
+        <v>23.22</v>
+      </c>
+      <c r="H75" s="11" t="n">
+        <v>61</v>
+      </c>
+      <c r="I75" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J75" s="11" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="12" t="n">
+        <v>73</v>
+      </c>
+      <c r="B76" s="12" t="inlineStr">
+        <is>
+          <t>(-0.00, -0.00)</t>
+        </is>
+      </c>
+      <c r="C76" s="12" t="inlineStr">
+        <is>
+          <t>(1.00, 3.01)</t>
+        </is>
+      </c>
+      <c r="D76" s="12" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E76" s="12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F76" s="12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G76" s="12" t="n">
+        <v>24.76</v>
+      </c>
+      <c r="H76" s="12" t="n">
+        <v>60</v>
+      </c>
+      <c r="I76" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J76" s="12" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="11" t="n">
+        <v>74</v>
+      </c>
+      <c r="B77" s="11" t="inlineStr">
+        <is>
+          <t>(-0.00, -0.00)</t>
+        </is>
+      </c>
+      <c r="C77" s="11" t="inlineStr">
+        <is>
+          <t>(0.99, 3.02)</t>
+        </is>
+      </c>
+      <c r="D77" s="11" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E77" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F77" s="11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G77" s="11" t="n">
+        <v>36.92</v>
+      </c>
+      <c r="H77" s="11" t="n">
+        <v>60</v>
+      </c>
+      <c r="I77" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J77" s="11" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="B78" s="12" t="inlineStr">
+        <is>
+          <t>(-0.00, -0.00)</t>
+        </is>
+      </c>
+      <c r="C78" s="12" t="inlineStr">
+        <is>
+          <t>(1.03, 3.02)</t>
+        </is>
+      </c>
+      <c r="D78" s="12" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E78" s="12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F78" s="12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G78" s="12" t="n">
+        <v>26.83</v>
+      </c>
+      <c r="H78" s="12" t="n">
+        <v>60</v>
+      </c>
+      <c r="I78" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J78" s="12" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="11" t="n">
+        <v>76</v>
+      </c>
+      <c r="B79" s="11" t="inlineStr">
+        <is>
+          <t>(-0.00, -0.00)</t>
+        </is>
+      </c>
+      <c r="C79" s="11" t="inlineStr">
+        <is>
+          <t>(1.00, 3.02)</t>
+        </is>
+      </c>
+      <c r="D79" s="11" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E79" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F79" s="11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G79" s="11" t="n">
+        <v>19.66</v>
+      </c>
+      <c r="H79" s="11" t="n">
+        <v>60</v>
+      </c>
+      <c r="I79" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J79" s="11" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="12" t="n">
+        <v>77</v>
+      </c>
+      <c r="B80" s="12" t="inlineStr">
+        <is>
+          <t>(-0.00, -0.00)</t>
+        </is>
+      </c>
+      <c r="C80" s="12" t="inlineStr">
+        <is>
+          <t>(1.02, 3.01)</t>
+        </is>
+      </c>
+      <c r="D80" s="12" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E80" s="12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F80" s="12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G80" s="12" t="n">
+        <v>20.73</v>
+      </c>
+      <c r="H80" s="12" t="n">
+        <v>60</v>
+      </c>
+      <c r="I80" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J80" s="12" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="11" t="n">
+        <v>78</v>
+      </c>
+      <c r="B81" s="11" t="inlineStr">
+        <is>
+          <t>(-0.00, -0.00)</t>
+        </is>
+      </c>
+      <c r="C81" s="11" t="inlineStr">
+        <is>
+          <t>(1.01, 3.03)</t>
+        </is>
+      </c>
+      <c r="D81" s="11" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E81" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F81" s="11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G81" s="11" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="H81" s="11" t="n">
+        <v>61</v>
+      </c>
+      <c r="I81" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J81" s="11" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>

</xml_diff>